<commit_message>
Add per-valve overhaul RH so overhaul-due counts hours since overhaul
Like unit decarbs, fuel/exhaust valve components now record when they
were last overhauled - both date and the component's running hours at
that overhaul:

- valve_components.last_overhaul_rh (nullable); when set, alert status
  everywhere (components list, valve dashboards, alerts, reports) is
  computed from RH since the overhaul instead of lifetime RH, and
  dashboard slot cards show hours since overhaul against the interval
- Add/Edit valve dialogs gain a "Last Overhaul" section with Overhaul
  Date and Overhauled-at-RH inputs
- Components table shows "at N hr" under the overhaul date and
  "N since O/H" under Live RH
- Excel import: new optional "Last Overhaul RH (hrs)" column on the
  valve sheets; sample template updated with examples
</commit_message>
<xml_diff>
--- a/artifacts/piston-rh/public/PistonRH_Import_Template.xlsx
+++ b/artifacts/piston-rh/public/PistonRH_Import_Template.xlsx
@@ -309,7 +309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -323,7 +323,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -331,7 +330,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -388,7 +386,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -403,7 +400,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -418,8 +414,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -448,7 +442,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -470,7 +463,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -478,7 +470,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -539,7 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -579,6 +569,20 @@
       <c r="A44" t="inlineStr">
         <is>
           <t xml:space="preserve">   overhauled. Leave blank if unknown. Format: YYYY-MM-DD (e.g. 2025-04-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>-  Valve sheets also take 'Last Overhaul RH (hrs)': the component's own running hours at its</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   last overhaul. When set, overhaul-due status counts hours run since that overhaul.</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1568,6 +1572,7 @@
     <col width="12.44140625" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="24.3" customHeight="1">
@@ -1625,6 +1630,12 @@
 (YYYY-MM-DD, optional)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Last Overhaul RH (hrs)
+(component RH at overhaul, optional)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="10.2" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -1754,6 +1765,9 @@
           <t>2025-04-05</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>5000</v>
+      </c>
     </row>
     <row r="5" ht="10.2" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -1797,6 +1811,9 @@
           <t>2025-04-06</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>5000</v>
+      </c>
     </row>
     <row r="6" ht="10.2" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -1883,6 +1900,9 @@
           <t>2025-04-08</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>550</v>
+      </c>
     </row>
     <row r="8" ht="10.2" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -1969,6 +1989,9 @@
           <t>2025-04-01</t>
         </is>
       </c>
+      <c r="K9" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="10" ht="10.2" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -2055,6 +2078,9 @@
           <t>2025-04-03</t>
         </is>
       </c>
+      <c r="K11" t="n">
+        <v>650</v>
+      </c>
     </row>
     <row r="12" ht="10.2" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -2140,6 +2166,9 @@
         <is>
           <t>2025-04-05</t>
         </is>
+      </c>
+      <c r="K13" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="14" ht="10.2" customHeight="1">
@@ -3548,7 +3577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3560,6 +3589,7 @@
     <col width="12.44140625" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="24.3" customHeight="1">
@@ -3617,6 +3647,12 @@
 (YYYY-MM-DD, optional)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Last Overhaul RH (hrs)
+(component RH at overhaul, optional)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="10.2" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -3703,6 +3739,9 @@
           <t>2025-02-13</t>
         </is>
       </c>
+      <c r="K3" t="n">
+        <v>700</v>
+      </c>
     </row>
     <row r="4" ht="10.2" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -3746,6 +3785,9 @@
           <t>2025-02-14</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>1050</v>
+      </c>
     </row>
     <row r="5" ht="10.2" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -3789,6 +3831,9 @@
           <t>2025-02-15</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>1400</v>
+      </c>
     </row>
     <row r="6" ht="10.2" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -3832,6 +3877,9 @@
           <t>2025-02-16</t>
         </is>
       </c>
+      <c r="K6" t="n">
+        <v>1750</v>
+      </c>
     </row>
     <row r="7" ht="10.2" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -3874,6 +3922,9 @@
         <is>
           <t>2025-02-17</t>
         </is>
+      </c>
+      <c r="K7" t="n">
+        <v>2100</v>
       </c>
     </row>
     <row r="8" ht="10.2" customHeight="1">

</xml_diff>

<commit_message>
Valve overhaul baseline is ME RH at overhaul, not component hours
Matches how crews actually record it (and the unit decarb convention):
the user enters the Main Engine total RH at which the fuel/exhaust
valve was overhauled, and hours-since-overhaul = current ME RH minus
that baseline - e.g. overhauled at ME 41,891, ME now 43,836 -> 1,945 of
the 8,000-hr interval.

- Dialogs relabelled "Overhauled at ME RH (hrs)"; table and dashboard
  cards show "at ME <N> hr"
- Sample template column note and example values updated to ME RH
- Added "Fuel Valve Body" and "Fuel Valve Spindle/Guide" to suggested
  fuel valve component types (the body is a child of the fuel valve
  with its own lifetime hours, like nozzle and spindle)
</commit_message>
<xml_diff>
--- a/artifacts/piston-rh/public/PistonRH_Import_Template.xlsx
+++ b/artifacts/piston-rh/public/PistonRH_Import_Template.xlsx
@@ -323,6 +323,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -330,6 +331,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -386,6 +388,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -400,6 +403,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -414,6 +418,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -442,6 +448,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -463,6 +470,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -470,6 +478,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -530,6 +539,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -537,6 +547,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
@@ -575,14 +586,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>-  Valve sheets also take 'Last Overhaul RH (hrs)': the component's own running hours at its</t>
+          <t>-  Valve sheets also take 'Last Overhaul RH (hrs)': the MAIN ENGINE total RH at which that</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   last overhaul. When set, overhaul-due status counts hours run since that overhaul.</t>
+          <t xml:space="preserve">   component was last overhauled. Overhaul-due status then counts ME hours run since that point.</t>
         </is>
       </c>
     </row>
@@ -683,6 +694,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="13.95" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
@@ -724,6 +736,7 @@
         <v>20000</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="13.95" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
@@ -767,6 +780,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="13.95" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
@@ -798,6 +812,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="13.95" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
@@ -1633,7 +1648,7 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Last Overhaul RH (hrs)
-(component RH at overhaul, optional)</t>
+(ME RH at overhaul, optional)</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1781,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>5000</v>
+        <v>14500</v>
       </c>
     </row>
     <row r="5" ht="10.2" customHeight="1">
@@ -1812,7 +1827,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>5000</v>
+        <v>13300</v>
       </c>
     </row>
     <row r="6" ht="10.2" customHeight="1">
@@ -1901,7 +1916,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>550</v>
+        <v>12100</v>
       </c>
     </row>
     <row r="8" ht="10.2" customHeight="1">
@@ -1990,7 +2005,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>600</v>
+        <v>10900</v>
       </c>
     </row>
     <row r="10" ht="10.2" customHeight="1">
@@ -2079,7 +2094,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>650</v>
+        <v>9700</v>
       </c>
     </row>
     <row r="12" ht="10.2" customHeight="1">
@@ -2168,7 +2183,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>700</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="14" ht="10.2" customHeight="1">
@@ -3650,7 +3665,7 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Last Overhaul RH (hrs)
-(component RH at overhaul, optional)</t>
+(ME RH at overhaul, optional)</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3755,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>700</v>
+        <v>14500</v>
       </c>
     </row>
     <row r="4" ht="10.2" customHeight="1">
@@ -3786,7 +3801,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>1050</v>
+        <v>13300</v>
       </c>
     </row>
     <row r="5" ht="10.2" customHeight="1">
@@ -3832,7 +3847,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>1400</v>
+        <v>12100</v>
       </c>
     </row>
     <row r="6" ht="10.2" customHeight="1">
@@ -3878,7 +3893,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>1750</v>
+        <v>10900</v>
       </c>
     </row>
     <row r="7" ht="10.2" customHeight="1">
@@ -3924,7 +3939,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>2100</v>
+        <v>9700</v>
       </c>
     </row>
     <row r="8" ht="10.2" customHeight="1">

</xml_diff>